<commit_message>
D-021 permission model; FSD v0.4; catalogue and tracker updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AzN61zWTi2yq5SJaQMPbTS
</commit_message>
<xml_diff>
--- a/docs/BEST_Clinic_User_Permissions_Catalogue.xlsx
+++ b/docs/BEST_Clinic_User_Permissions_Catalogue.xlsx
@@ -115,7 +115,7 @@
     <t xml:space="preserve">Agreed</t>
   </si>
   <si>
-    <t xml:space="preserve">FSD v0.3 S5; PRD 8.1</t>
+    <t xml:space="preserve">FSD v0.4 S5; PRD 8.1</t>
   </si>
   <si>
     <t xml:space="preserve">ACC-02</t>
@@ -127,7 +127,7 @@
     <t xml:space="preserve">Set a new password at first login; reset through Forgot password</t>
   </si>
   <si>
-    <t xml:space="preserve">FSD v0.3 S6, S8</t>
+    <t xml:space="preserve">FSD v0.4 S6, S8</t>
   </si>
   <si>
     <t xml:space="preserve">ACC-03</t>
@@ -142,7 +142,7 @@
     <t xml:space="preserve">MFA on for the user</t>
   </si>
   <si>
-    <t xml:space="preserve">FSD v0.3 S7, BR-11</t>
+    <t xml:space="preserve">FSD v0.4 S7, BR-11</t>
   </si>
   <si>
     <t xml:space="preserve">ACC-04</t>
@@ -820,7 +820,7 @@
     <t xml:space="preserve">Trends across a client’s sessions</t>
   </si>
   <si>
-    <t xml:space="preserve">FSD v0.3 role defaults</t>
+    <t xml:space="preserve">FSD v0.4 role defaults</t>
   </si>
   <si>
     <t xml:space="preserve">RPT-02</t>
@@ -865,7 +865,7 @@
     <t xml:space="preserve">Users, roles, status, last login</t>
   </si>
   <si>
-    <t xml:space="preserve">FSD v0.3 S1</t>
+    <t xml:space="preserve">FSD v0.4 S1</t>
   </si>
   <si>
     <t xml:space="preserve">USR-02</t>
@@ -883,7 +883,7 @@
     <t xml:space="preserve">Active-user limit</t>
   </si>
   <si>
-    <t xml:space="preserve">FSD v0.3 S2–S3</t>
+    <t xml:space="preserve">FSD v0.4 S2–S3</t>
   </si>
   <si>
     <t xml:space="preserve">USR-03</t>
@@ -895,7 +895,7 @@
     <t xml:space="preserve">View or Edit on Users &amp; roles or Clinic settings</t>
   </si>
   <si>
-    <t xml:space="preserve">FSD v0.3 BR-18</t>
+    <t xml:space="preserve">FSD v0.4 BR-18</t>
   </si>
   <si>
     <t xml:space="preserve">USR-04</t>
@@ -907,7 +907,7 @@
     <t xml:space="preserve">Off by default</t>
   </si>
   <si>
-    <t xml:space="preserve">FSD v0.3 S3, BR-11</t>
+    <t xml:space="preserve">FSD v0.4 S3, BR-11</t>
   </si>
   <si>
     <t xml:space="preserve">USR-05</t>
@@ -919,7 +919,7 @@
     <t xml:space="preserve">After creation; permissions come from the role</t>
   </si>
   <si>
-    <t xml:space="preserve">PRD 8.9 (out of FSD v0.3 scope)</t>
+    <t xml:space="preserve">PRD 8.9 (out of FSD v0.4 scope)</t>
   </si>
   <si>
     <t xml:space="preserve">USR-06</t>
@@ -931,7 +931,7 @@
     <t xml:space="preserve">Blocks login; stops counting as an active user</t>
   </si>
   <si>
-    <t xml:space="preserve">FSD v0.3 S9, BR-18</t>
+    <t xml:space="preserve">FSD v0.4 S9, BR-18</t>
   </si>
   <si>
     <t xml:space="preserve">USR-07</t>
@@ -943,7 +943,7 @@
     <t xml:space="preserve">If the active-user limit allows</t>
   </si>
   <si>
-    <t xml:space="preserve">FSD v0.3 S9</t>
+    <t xml:space="preserve">FSD v0.4 S9</t>
   </si>
   <si>
     <t xml:space="preserve">USR-08</t>
@@ -955,7 +955,7 @@
     <t xml:space="preserve">New temporary password</t>
   </si>
   <si>
-    <t xml:space="preserve">FSD v0.3 BR-09</t>
+    <t xml:space="preserve">FSD v0.4 BR-09</t>
   </si>
   <si>
     <t xml:space="preserve">USR-09</t>
@@ -970,7 +970,7 @@
     <t xml:space="preserve">When the role has admin modules</t>
   </si>
   <si>
-    <t xml:space="preserve">FSD v0.3 S4, BR-18</t>
+    <t xml:space="preserve">FSD v0.4 S4, BR-18</t>
   </si>
   <si>
     <t xml:space="preserve">USR-10</t>
@@ -982,7 +982,7 @@
     <t xml:space="preserve">Edits apply to every user holding the role; a role in use cannot be retired</t>
   </si>
   <si>
-    <t xml:space="preserve">FSD v0.3 S4, S12; BR-23, BR-24</t>
+    <t xml:space="preserve">FSD v0.4 S4, S12; BR-23, BR-24</t>
   </si>
   <si>
     <t xml:space="preserve">USR-11</t>
@@ -994,7 +994,7 @@
     <t xml:space="preserve">Predefined and custom roles with their modules (S12)</t>
   </si>
   <si>
-    <t xml:space="preserve">FSD v0.3 2.2, S12</t>
+    <t xml:space="preserve">FSD v0.4 2.2, S12</t>
   </si>
   <si>
     <t xml:space="preserve">Clinic settings  ·  9 permissions</t>
@@ -1039,7 +1039,7 @@
     <t xml:space="preserve">Text, number, date or dropdown; optional or mandatory</t>
   </si>
   <si>
-    <t xml:space="preserve">FSD v0.3 S2</t>
+    <t xml:space="preserve">FSD v0.4 S2</t>
   </si>
   <si>
     <t xml:space="preserve">SET-05</t>
@@ -1108,7 +1108,7 @@
     <t xml:space="preserve">Logins, user and role changes, consent and client changes</t>
   </si>
   <si>
-    <t xml:space="preserve">FSD v0.3 Section 10</t>
+    <t xml:space="preserve">FSD v0.4 Section 10</t>
   </si>
   <si>
     <t xml:space="preserve">AUD-02</t>
@@ -1210,7 +1210,7 @@
     <t xml:space="preserve">SPV, DEV, SUP rows</t>
   </si>
   <si>
-    <t xml:space="preserve">Yes; they cover features already agreed</t>
+    <t xml:space="preserve">Decided 28 Oct (D-021): added; 14 modules in FSD v0.4. Awaiting BEST confirmation</t>
   </si>
   <si>
     <t xml:space="preserve">Should anyone download attachments, export reports or export the audit log?</t>
@@ -1258,22 +1258,22 @@
     <t xml:space="preserve">Merge: keep IDs, take role defaults from the RBAC list</t>
   </si>
   <si>
-    <t xml:space="preserve">FSD v0.3 sets permissions per module (None, View or Edit). That cannot express some defaults here, e.g. a supervisor who views sessions but also creates them. Switch the Create user and Create role screens to permission-level ticks grouped by module?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FSD v0.3 S3, S4; all rows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yes: ticks per permission, with a module-level ‘select all’</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FSD v0.3 gives the Org Admin no Sessions access, but the agreed Org Admin flow (D-014) has the Org Admin scheduling sessions. Allow scheduling only (SES-01 to SES-05), with no session content?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SES-01 to SES-05; FSD v0.3 2.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yes: schedule only; session records stay hidden</t>
+    <t xml:space="preserve">Should roles be built per module (None, View or Edit) or by ticking individual permissions?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FSD S3, S4; all rows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decided 28 Oct (D-021): ticks per permission, grouped by module, with Select all and a scope per permission (FSD v0.4 S4, BR-26). Awaiting BEST confirmation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Should the Org Admin role schedule sessions without seeing session content?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SES-01 to SES-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decided 28 Oct (D-021): scheduling only (SES-01 to SES-05); session records stay hidden (FSD v0.4 §2.2). Awaiting BEST confirmation</t>
   </si>
 </sst>
 </file>
@@ -7951,7 +7951,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="116" t="n">
         <v>4</v>
       </c>
@@ -8049,7 +8049,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="116" t="n">
         <v>11</v>
       </c>

</xml_diff>